<commit_message>
Refactor API data fetching and enhance multi-game support
- Improved the `_get_json` function for better error handling and code reuse across various fetch modules.
- Updated the User-Agent in fetch requests to enhance compatibility with external APIs.
- Added new CLI commands for fetching additional game data, including Bandai JP One Piece.
- Expanded sports seed data in `data/raw/sports/seed.json` to include more manufacturers and sports.
- Updated documentation to reflect recent changes and clarify the data fetching process.

This commit enhances the API's functionality and improves the user experience for multi-game support.
</commit_message>
<xml_diff>
--- a/sources/sports_cards.xlsx
+++ b/sources/sports_cards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,11 +469,7 @@
           <t>2025-26-topps-manchester-united-team-set</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-26 TOPPS MANCHESTER UNITED TEAM SET</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>38</t>
@@ -500,11 +496,7 @@
           <t>2025-26-topps-manchester-united-team-set</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2025-26 TOPPS MANCHESTER UNITED TEAM SET</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>38</t>
@@ -532,22 +524,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-panini-flawless-wwe</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2024 PANINI FLAWLESS WWE</t>
-        </is>
-      </c>
+          <t>2025-26-topps-manchester-united-team-set</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SSL-SM</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SHAWN MICHAELS</t>
+          <t>CRISTIANO RONALDO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -556,54 +544,1255 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>SHAWN MICHAELS</t>
+          <t>CRISTIANO RONALDO</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>2025-26-topps-manchester-united-team-set</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CRISTIANO RONALDO</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GOLD PARALLEL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CRISTIANO RONALDO - GOLD PARALLEL - 25/50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-26-topps-manchester-united-team-set</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>MARCUS RASHFORD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BLUE REFRACTOR</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>MARCUS RASHFORD - BLUE REFRACTOR - 49/150</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-26-topps-manchester-united-team-set</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ALEJANDRO GARNACHO</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ALEJANDRO GARNACHO - RC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>2024-panini-flawless-wwe</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2024 PANINI FLAWLESS WWE</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
         <is>
           <t>SSL-SM</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>SHAWN MICHAELS</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>SHAWN MICHAELS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2024-panini-flawless-wwe</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SSL-SM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SHAWN MICHAELS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>RUBY REF</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H9" t="n">
+        <v>15</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>SHAWN MICHAELS – AUTO - RUBY REF. – 09/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2024-panini-flawless-wwe</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SSL-UA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>THE UNDERTAKER</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DIAMOND</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>10</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>THE UNDERTAKER – AUTO - DIAMOND – 03/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2024-panini-flawless-wwe</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SSL-JC</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>JOHN CENA</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>EMERALD</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>JOHN CENA – AUTO - EMERALD – 04/5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-topps-chrome-football</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PATRICK MAHOMES</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>PATRICK MAHOMES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-topps-chrome-football</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PATRICK MAHOMES</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>REFRACTOR</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>PATRICK MAHOMES - REFRACTOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-topps-chrome-football</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CJ STROUD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>CJ STROUD - RC</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-topps-chrome-football</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CJ STROUD</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ORANGE REFRACTOR</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>25</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>CJ STROUD - RC - ORANGE REFRACTOR - 18/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-topps-chrome-football</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>JALEN HURTS</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PURPLE REFRACTOR</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>75</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>JALEN HURTS - PURPLE REFRACTOR - 22/75</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-upper-deck-aew-wrestling</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CM PUNK</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>CM PUNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-upper-deck-aew-wrestling</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CM PUNK</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BLUE PARALLEL</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>CM PUNK - BLUE PARALLEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-upper-deck-aew-wrestling</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MJF</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>25</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>MJF - AUTO - GOLD - 05/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-upper-deck-aew-wrestling</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>WILL OSPREAY</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>25</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>WILL OSPREAY - AUTO - RED - 11/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2024-panini-prizm-soccer</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>LIONEL MESSI</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>LIONEL MESSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2024-panini-prizm-soccer</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>LIONEL MESSI</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SILVER PRIZM</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LIONEL MESSI - SILVER PRIZM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2024-panini-prizm-soccer</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KYLIAN MBAPPE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>GREEN WAVE</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>99</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>KYLIAN MBAPPE - GREEN WAVE - 12/99</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2024-panini-prizm-soccer</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ERLING HAALAND</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>GOLD PRIZM</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>10</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ERLING HAALAND - GOLD PRIZM - 07/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1996-97-skybox-premium-basketball</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MICHAEL JORDAN</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>MICHAEL JORDAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1996-97-skybox-premium-basketball</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>SHAWN MICHAELS – AUTO - RUBY REF. – 09/15</t>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>KOBE BRYANT</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>KOBE BRYANT - RC</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1996-97-skybox-premium-basketball</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ALLEN IVERSON</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>ALLEN IVERSON - RC</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2024-topps-chrome-ufc</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CONOR MCGREGOR</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>CONOR MCGREGOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2024-topps-chrome-ufc</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CONOR MCGREGOR</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>GOLD REFRACTOR</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>50</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>CONOR MCGREGOR - GOLD REFRACTOR - 08/50</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2024-topps-chrome-ufc</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ISLAM MAKHACHEV</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BLUE WAVE</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>75</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>ISLAM MAKHACHEV - AUTO - BLUE WAVE - 14/75</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2024-topps-chrome-ufc</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ALEXANDER VOLKANOVSKI</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>REFRACTOR</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>ALEXANDER VOLKANOVSKI - REFRACTOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2024-panini-donruss-football</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>JOSH ALLEN</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>JOSH ALLEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2024-panini-donruss-football</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>JOSH ALLEN</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>RATED ROOKIE OPTIC</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>JOSH ALLEN - RATED ROOKIE OPTIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2024-panini-donruss-football</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>308</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CALEB WILLIAMS</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>RATED ROOKIE</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>CALEB WILLIAMS - RC - RATED ROOKIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-topps-uefa-club-competitions</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>VINICIUS JUNIOR</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>VINICIUS JUNIOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-topps-uefa-club-competitions</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>VINICIUS JUNIOR</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>GOLD FOIL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>50</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>VINICIUS JUNIOR - GOLD FOIL - 10/50</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-topps-uefa-club-competitions</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>JUDE BELLINGHAM</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>AQUA PARALLEL</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>99</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>JUDE BELLINGHAM - AQUA PARALLEL - 33/99</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1989-bandai-carddass-dbz-part1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>孫悟空</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>孫悟空</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1989-bandai-carddass-dbz-part1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>フリーザ</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>フリーザ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1998-meiji-pokemon-get-card</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>ピカチュウ</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>ピカチュウ</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1992-marvel-universe-series-1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>SPIDER-MAN</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>SPIDER-MAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1992-marvel-universe-series-1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>WOLVERINE</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>WOLVERINE</t>
         </is>
       </c>
     </row>

</xml_diff>